<commit_message>
Did some work, cleared up why data-theme is a superior approach to suffix based theme dependant styling, will continue using data-theme approach in the future and will also teach myself how to implement it better
</commit_message>
<xml_diff>
--- a/docs/TODO.xlsx
+++ b/docs/TODO.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\WebstormProjects\fakeStore\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tynek\WebstormProjects\fakeStore\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE2BC168-B765-4151-BCEB-78202B353EB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D113BCC0-4F20-4FBE-A6C6-FC74BE1BFC3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12396" yWindow="0" windowWidth="10740" windowHeight="12336" xr2:uid="{34F18800-7D7C-49F0-9E38-8C232BBC83B4}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{34F18800-7D7C-49F0-9E38-8C232BBC83B4}"/>
   </bookViews>
   <sheets>
     <sheet name="TODO" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -175,7 +176,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -511,220 +512,220 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF0C54FF-8834-4BD0-B801-E6897FE41320}">
-  <dimension ref="B4:C29"/>
+  <dimension ref="C2:D27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="5.5546875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="70.5546875" style="2" customWidth="1"/>
-    <col min="4" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="2" width="8.88671875" style="1"/>
+    <col min="3" max="3" width="3" style="3" customWidth="1"/>
+    <col min="4" max="4" width="70.5546875" style="2" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B4" s="3">
+    <row r="2" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C2" s="3">
         <v>1</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B5" s="3">
+    <row r="3" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C3" s="3">
         <v>2</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B6" s="3">
+    <row r="4" spans="3:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C4" s="3">
         <v>3</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B7" s="3">
+    <row r="5" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C5" s="3">
         <v>4</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B8" s="3">
+    <row r="6" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C6" s="3">
         <v>5</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B9" s="3">
+    <row r="7" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C7" s="3">
         <v>6</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B10" s="3">
+    <row r="8" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C8" s="3">
         <v>7</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B11" s="3">
+    <row r="9" spans="3:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C9" s="3">
         <v>8</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B12" s="3">
+    <row r="10" spans="3:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C10" s="3">
         <v>9</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B13" s="3">
+    <row r="11" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C11" s="3">
         <v>10</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B14" s="3">
+    <row r="12" spans="3:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C12" s="3">
         <v>11</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B15" s="3">
+    <row r="13" spans="3:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C13" s="3">
         <v>12</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B16" s="3">
+    <row r="14" spans="3:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C14" s="3">
         <v>13</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B17" s="3">
+    <row r="15" spans="3:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C15" s="3">
         <v>14</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B18" s="3">
+    <row r="16" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C16" s="3">
         <v>15</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B19" s="3">
+    <row r="17" spans="3:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C17" s="3">
         <v>16</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B20" s="3">
+    <row r="18" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C18" s="3">
         <v>17</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B21" s="3">
+    <row r="19" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C19" s="3">
         <v>18</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B22" s="3">
+    <row r="20" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C20" s="3">
         <v>19</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B23" s="3">
+    <row r="21" spans="3:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C21" s="3">
         <v>20</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B24" s="3">
+    <row r="22" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C22" s="3">
         <v>21</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B25" s="3">
+    <row r="23" spans="3:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C23" s="3">
         <v>22</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="D23" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B26" s="3">
+    <row r="24" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C24" s="3">
         <v>23</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="2:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B27" s="3">
+    <row r="25" spans="3:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C25" s="3">
         <v>24</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="D25" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B28" s="3">
+    <row r="26" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C26" s="3">
         <v>25</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="D26" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B29" s="3">
+    <row r="27" spans="3:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C27" s="3">
         <v>26</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>